<commit_message>
feat: add prev fev-abr 2026
</commit_message>
<xml_diff>
--- a/data/accb_custo_total_ilheus.xlsx
+++ b/data/accb_custo_total_ilheus.xlsx
@@ -39,12 +39,10 @@
     </font>
     <font>
       <sz val="10.000000"/>
-      <color indexed="64"/>
       <name val="Calibri"/>
     </font>
     <font>
       <sz val="11.000000"/>
-      <color indexed="64"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -2600,8 +2598,12 @@
       </c>
     </row>
     <row r="254" ht="15.75" customHeight="1">
-      <c r="A254" s="7"/>
-      <c r="B254" s="5"/>
+      <c r="A254" s="7">
+        <v>46023</v>
+      </c>
+      <c r="B254" s="5">
+        <v>553.40999999999997</v>
+      </c>
     </row>
     <row r="255" ht="15.75" customHeight="1">
       <c r="A255" s="7"/>

</xml_diff>

<commit_message>
feat: add prev mar-mai 2026 fix: refatoração funções projeto
</commit_message>
<xml_diff>
--- a/data/accb_custo_total_ilheus.xlsx
+++ b/data/accb_custo_total_ilheus.xlsx
@@ -2606,8 +2606,12 @@
       </c>
     </row>
     <row r="255" ht="15.75" customHeight="1">
-      <c r="A255" s="7"/>
-      <c r="B255" s="5"/>
+      <c r="A255" s="7">
+        <v>46054</v>
+      </c>
+      <c r="B255" s="5">
+        <v>565.25999999999999</v>
+      </c>
     </row>
     <row r="256" ht="15.75" customHeight="1">
       <c r="A256" s="7"/>

</xml_diff>